<commit_message>
Adiciona conciliação de caixinhas RDB e reincluiu aplicações nas saídas
- Nova aba CONCILIAÇÃO CAIXINHAS com extrato completo do RDB
- Cruza cada aplicação do extrato bancário com compras no extrato de caixinhas
- Mostra rendimentos acumulados, resgates e saldo final R$ 68.284,51
- Reincluiu saídas para aplicação RDB na aba de pagamentos e fluxo de caixa

https://claude.ai/code/session_01G5mMjRFfSUYsTe2acKL7Qd
</commit_message>
<xml_diff>
--- a/CONCILIACAO_COMPLETA_2024_2026.xlsx
+++ b/CONCILIACAO_COMPLETA_2024_2026.xlsx
@@ -13,6 +13,7 @@
     <sheet name="FLUXO DE CAIXA" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="DETALHE ENTRADAS" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="DIVERGÊNCIAS" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="CONCILIAÇÃO CAIXINHAS" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -24,7 +25,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="16">
+  <fonts count="20">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -95,8 +96,26 @@
       <b val="1"/>
       <color rgb="00FF0000"/>
     </font>
+    <font>
+      <color rgb="00C00000"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00006100"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00C00000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00C00000"/>
+      <sz val="13"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -145,6 +164,24 @@
         <bgColor rgb="00C00000"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00548235"/>
+        <bgColor rgb="00548235"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+        <bgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
+        <bgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -164,7 +201,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -221,11 +258,33 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="13" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="15" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="16" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="17" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="18" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="9" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -5951,7 +6010,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:E61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -5971,7 +6030,7 @@
     <row r="2">
       <c r="A2" s="28" t="inlineStr">
         <is>
-          <t>Total de saídas: R$ 55,211.92</t>
+          <t>Total de saídas: R$ 159,793.45</t>
         </is>
       </c>
     </row>
@@ -6005,75 +6064,75 @@
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>23/07/2024</t>
+          <t>15/07/2024</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>BOLETO</t>
+          <t>APLICAÇÃO RDB</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>IBIUNA</t>
+          <t>Investimento automático</t>
         </is>
       </c>
       <c r="D5" s="9" t="n">
-        <v>45.1</v>
+        <v>8800</v>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>PREFEITURA/CARTÓRIO</t>
+          <t>APLICAÇÃO RDB</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>23/07/2024</t>
+          <t>16/07/2024</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>BOLETO</t>
+          <t>APLICAÇÃO RDB</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>IBIUNA</t>
+          <t>Investimento automático</t>
         </is>
       </c>
       <c r="D6" s="9" t="n">
-        <v>45.1</v>
+        <v>500</v>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>PREFEITURA/CARTÓRIO</t>
+          <t>APLICAÇÃO RDB</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>23/07/2024</t>
+          <t>21/07/2024</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>BOLETO</t>
+          <t>APLICAÇÃO RDB</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>IBIUNA</t>
+          <t>Investimento automático</t>
         </is>
       </c>
       <c r="D7" s="9" t="n">
-        <v>135.32</v>
+        <v>1500</v>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>PREFEITURA/CARTÓRIO</t>
+          <t>APLICAÇÃO RDB</t>
         </is>
       </c>
     </row>
@@ -6119,7 +6178,7 @@
         </is>
       </c>
       <c r="D9" s="9" t="n">
-        <v>135.32</v>
+        <v>45.1</v>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
@@ -6130,82 +6189,82 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>24/07/2024</t>
+          <t>23/07/2024</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>PIX ENVIADO</t>
+          <t>BOLETO</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Cesar Augusto de Oliveira</t>
+          <t>IBIUNA</t>
         </is>
       </c>
       <c r="D10" s="9" t="n">
-        <v>3000</v>
+        <v>135.32</v>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>PIX P/ TERCEIROS</t>
+          <t>PREFEITURA/CARTÓRIO</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>24/07/2024</t>
+          <t>23/07/2024</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>PIX ENVIADO</t>
+          <t>BOLETO</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>MARINA LEITE AGOSTINHO SOCIEDADE</t>
+          <t>IBIUNA</t>
         </is>
       </c>
       <c r="D11" s="9" t="n">
-        <v>6000</v>
+        <v>45.1</v>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>HONORÁRIOS</t>
+          <t>PREFEITURA/CARTÓRIO</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>27/08/2024</t>
+          <t>23/07/2024</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>PIX ENVIADO</t>
+          <t>BOLETO</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Marina Leite Agostinho Sociedade Individual de</t>
+          <t>IBIUNA</t>
         </is>
       </c>
       <c r="D12" s="9" t="n">
-        <v>9000</v>
+        <v>135.32</v>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>HONORÁRIOS</t>
+          <t>PREFEITURA/CARTÓRIO</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>21/09/2024</t>
+          <t>24/07/2024</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
@@ -6215,11 +6274,11 @@
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>ALISSON RAFAEL MORAES</t>
+          <t>Cesar Augusto de Oliveira</t>
         </is>
       </c>
       <c r="D13" s="9" t="n">
-        <v>35.36</v>
+        <v>3000</v>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
@@ -6230,7 +6289,7 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>10/10/2024</t>
+          <t>24/07/2024</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
@@ -6240,147 +6299,147 @@
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>Editora Ibiuna Ltda</t>
+          <t>MARINA LEITE AGOSTINHO SOCIEDADE</t>
         </is>
       </c>
       <c r="D14" s="9" t="n">
-        <v>190</v>
+        <v>6000</v>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>PREFEITURA/CARTÓRIO</t>
+          <t>HONORÁRIOS</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>13/10/2024</t>
+          <t>06/08/2024</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>PIX ENVIADO</t>
+          <t>APLICAÇÃO RDB</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>WANIA CRISTINA DA CRUZ</t>
+          <t>Investimento automático</t>
         </is>
       </c>
       <c r="D15" s="9" t="n">
-        <v>138.69</v>
+        <v>594.16</v>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>PIX P/ TERCEIROS</t>
+          <t>APLICAÇÃO RDB</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>23/10/2024</t>
+          <t>11/08/2024</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>PIX ENVIADO</t>
+          <t>APLICAÇÃO RDB</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>Dionisio Grangeiro Neto</t>
+          <t>Investimento automático</t>
         </is>
       </c>
       <c r="D16" s="9" t="n">
-        <v>4950</v>
+        <v>6000</v>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>TOPÓGRAFO</t>
+          <t>APLICAÇÃO RDB</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>17/01/2025</t>
+          <t>13/08/2024</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>PIX ENVIADO</t>
+          <t>APLICAÇÃO RDB</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>Dionisio Grangeiro Neto</t>
+          <t>Investimento automático</t>
         </is>
       </c>
       <c r="D17" s="9" t="n">
-        <v>11900</v>
+        <v>500</v>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>TOPÓGRAFO</t>
+          <t>APLICAÇÃO RDB</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>17/03/2025</t>
+          <t>18/08/2024</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>PIX ENVIADO</t>
+          <t>APLICAÇÃO RDB</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>DIONISIO GRANGEIRO NETO</t>
+          <t>Investimento automático</t>
         </is>
       </c>
       <c r="D18" s="9" t="n">
-        <v>11900</v>
+        <v>1000</v>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>TOPÓGRAFO</t>
+          <t>APLICAÇÃO RDB</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>22/04/2025</t>
+          <t>25/08/2024</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>PIX ENVIADO</t>
+          <t>APLICAÇÃO RDB</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>Gicele Capovilla Alves</t>
+          <t>Investimento automático</t>
         </is>
       </c>
       <c r="D19" s="9" t="n">
-        <v>3800</v>
+        <v>1500</v>
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>PIX P/ TERCEIROS</t>
+          <t>APLICAÇÃO RDB</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>01/07/2025</t>
+          <t>27/08/2024</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
@@ -6390,47 +6449,47 @@
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>JOSE OGIER JACOM NETO</t>
+          <t>Marina Leite Agostinho Sociedade Individual de</t>
         </is>
       </c>
       <c r="D20" s="9" t="n">
-        <v>1750</v>
+        <v>9000</v>
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>PIX P/ TERCEIROS</t>
+          <t>HONORÁRIOS</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>06/11/2025</t>
+          <t>16/09/2024</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>PIX ENVIADO</t>
+          <t>APLICAÇÃO RDB</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>SIMONE BASTOS GOMES</t>
+          <t>Investimento automático</t>
         </is>
       </c>
       <c r="D21" s="9" t="n">
-        <v>196.43</v>
+        <v>6000</v>
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>PIX P/ TERCEIROS</t>
+          <t>APLICAÇÃO RDB</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>10/11/2025</t>
+          <t>21/09/2024</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
@@ -6440,11 +6499,11 @@
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>Simone Bastos Gomes</t>
+          <t>ALISSON RAFAEL MORAES</t>
         </is>
       </c>
       <c r="D22" s="9" t="n">
-        <v>1750</v>
+        <v>35.36</v>
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
@@ -6455,21 +6514,21 @@
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>09/02/2026</t>
+          <t>10/10/2024</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>BOLETO</t>
+          <t>PIX ENVIADO</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>GEAZI ASSIS DE SOUZA OLIVEIRA</t>
+          <t>Editora Ibiuna Ltda</t>
         </is>
       </c>
       <c r="D23" s="9" t="n">
-        <v>195.5</v>
+        <v>190</v>
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
@@ -6477,107 +6536,823 @@
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>13/10/2024</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>PIX ENVIADO</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>WANIA CRISTINA DA CRUZ</t>
+        </is>
+      </c>
+      <c r="D24" s="9" t="n">
+        <v>138.69</v>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>PIX P/ TERCEIROS</t>
+        </is>
+      </c>
+    </row>
     <row r="25">
-      <c r="C25" s="28" t="inlineStr">
-        <is>
-          <t>TOTAL GERAL</t>
-        </is>
-      </c>
-      <c r="D25" s="30" t="n">
-        <v>55211.92000000001</v>
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>13/10/2024</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>APLICAÇÃO RDB</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>Investimento automático</t>
+        </is>
+      </c>
+      <c r="D25" s="9" t="n">
+        <v>7635.95</v>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>APLICAÇÃO RDB</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>23/10/2024</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>PIX ENVIADO</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>Dionisio Grangeiro Neto</t>
+        </is>
+      </c>
+      <c r="D26" s="9" t="n">
+        <v>4950</v>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>TOPÓGRAFO</t>
+        </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="31" t="inlineStr">
-        <is>
-          <t>RESUMO POR CATEGORIA</t>
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>30/10/2024</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>APLICAÇÃO RDB</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>Investimento automático</t>
+        </is>
+      </c>
+      <c r="D27" s="9" t="n">
+        <v>500</v>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>APLICAÇÃO RDB</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="32" t="inlineStr">
-        <is>
-          <t>CATEGORIA</t>
-        </is>
-      </c>
-      <c r="B28" s="32" t="inlineStr">
-        <is>
-          <t>QTD</t>
-        </is>
-      </c>
-      <c r="C28" s="32" t="inlineStr">
-        <is>
-          <t>TOTAL (R$)</t>
-        </is>
-      </c>
-      <c r="D28" s="32" t="inlineStr">
-        <is>
-          <t>%</t>
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>24/11/2024</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>APLICAÇÃO RDB</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>Investimento automático</t>
+        </is>
+      </c>
+      <c r="D28" s="9" t="n">
+        <v>7250</v>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>APLICAÇÃO RDB</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>HONORÁRIOS</t>
-        </is>
-      </c>
-      <c r="B29" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="C29" s="33" t="n">
-        <v>15000</v>
-      </c>
-      <c r="D29" s="34" t="n">
-        <v>0.2716804632043225</v>
+          <t>06/01/2025</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>APLICAÇÃO RDB</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>Investimento automático</t>
+        </is>
+      </c>
+      <c r="D29" s="9" t="n">
+        <v>7000</v>
+      </c>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>APLICAÇÃO RDB</t>
+        </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>TOPÓGRAFO</t>
-        </is>
-      </c>
-      <c r="B30" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="C30" s="33" t="n">
-        <v>28750</v>
-      </c>
-      <c r="D30" s="34" t="n">
-        <v>0.5207208878082848</v>
+          <t>07/01/2025</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>APLICAÇÃO RDB</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>Investimento automático</t>
+        </is>
+      </c>
+      <c r="D30" s="9" t="n">
+        <v>250</v>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>APLICAÇÃO RDB</t>
+        </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>PREFEITURA/CARTÓRIO</t>
-        </is>
-      </c>
-      <c r="B31" s="5" t="n">
-        <v>7</v>
-      </c>
-      <c r="C31" s="33" t="n">
-        <v>791.4400000000001</v>
-      </c>
-      <c r="D31" s="34" t="n">
-        <v>0.01433458571989527</v>
+          <t>12/01/2025</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>APLICAÇÃO RDB</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>Investimento automático</t>
+        </is>
+      </c>
+      <c r="D31" s="9" t="n">
+        <v>1250</v>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>APLICAÇÃO RDB</t>
+        </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
+          <t>17/01/2025</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>PIX ENVIADO</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>Dionisio Grangeiro Neto</t>
+        </is>
+      </c>
+      <c r="D32" s="9" t="n">
+        <v>11900</v>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>TOPÓGRAFO</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>02/02/2025</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>APLICAÇÃO RDB</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>Investimento automático</t>
+        </is>
+      </c>
+      <c r="D33" s="9" t="n">
+        <v>1500</v>
+      </c>
+      <c r="E33" s="5" t="inlineStr">
+        <is>
+          <t>APLICAÇÃO RDB</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>23/02/2025</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>APLICAÇÃO RDB</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>Investimento automático</t>
+        </is>
+      </c>
+      <c r="D34" s="9" t="n">
+        <v>3250</v>
+      </c>
+      <c r="E34" s="5" t="inlineStr">
+        <is>
+          <t>APLICAÇÃO RDB</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>16/03/2025</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>APLICAÇÃO RDB</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>Investimento automático</t>
+        </is>
+      </c>
+      <c r="D35" s="9" t="n">
+        <v>3250</v>
+      </c>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>APLICAÇÃO RDB</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>17/03/2025</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>PIX ENVIADO</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>DIONISIO GRANGEIRO NETO</t>
+        </is>
+      </c>
+      <c r="D36" s="9" t="n">
+        <v>11900</v>
+      </c>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>TOPÓGRAFO</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>12/04/2025</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>APLICAÇÃO RDB</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>Investimento automático</t>
+        </is>
+      </c>
+      <c r="D37" s="9" t="n">
+        <v>2750</v>
+      </c>
+      <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>APLICAÇÃO RDB</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>22/04/2025</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>PIX ENVIADO</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>Gicele Capovilla Alves</t>
+        </is>
+      </c>
+      <c r="D38" s="9" t="n">
+        <v>3800</v>
+      </c>
+      <c r="E38" s="5" t="inlineStr">
+        <is>
           <t>PIX P/ TERCEIROS</t>
         </is>
       </c>
-      <c r="B32" s="5" t="n">
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>15/06/2025</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>APLICAÇÃO RDB</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>Investimento automático</t>
+        </is>
+      </c>
+      <c r="D39" s="9" t="n">
+        <v>10251.42</v>
+      </c>
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>APLICAÇÃO RDB</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>01/07/2025</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>PIX ENVIADO</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>JOSE OGIER JACOM NETO</t>
+        </is>
+      </c>
+      <c r="D40" s="9" t="n">
+        <v>1750</v>
+      </c>
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>PIX P/ TERCEIROS</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>08/08/2025</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>APLICAÇÃO RDB</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>Investimento automático</t>
+        </is>
+      </c>
+      <c r="D41" s="9" t="n">
+        <v>3750</v>
+      </c>
+      <c r="E41" s="5" t="inlineStr">
+        <is>
+          <t>APLICAÇÃO RDB</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>11/08/2025</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>APLICAÇÃO RDB</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>Investimento automático</t>
+        </is>
+      </c>
+      <c r="D42" s="9" t="n">
+        <v>2250</v>
+      </c>
+      <c r="E42" s="5" t="inlineStr">
+        <is>
+          <t>APLICAÇÃO RDB</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>08/09/2025</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>APLICAÇÃO RDB</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>Investimento automático</t>
+        </is>
+      </c>
+      <c r="D43" s="9" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E43" s="5" t="inlineStr">
+        <is>
+          <t>APLICAÇÃO RDB</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>12/10/2025</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t>APLICAÇÃO RDB</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>Investimento automático</t>
+        </is>
+      </c>
+      <c r="D44" s="9" t="n">
+        <v>6500</v>
+      </c>
+      <c r="E44" s="5" t="inlineStr">
+        <is>
+          <t>APLICAÇÃO RDB</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>06/11/2025</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>PIX ENVIADO</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>SIMONE BASTOS GOMES</t>
+        </is>
+      </c>
+      <c r="D45" s="9" t="n">
+        <v>196.43</v>
+      </c>
+      <c r="E45" s="5" t="inlineStr">
+        <is>
+          <t>PIX P/ TERCEIROS</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>10/11/2025</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="inlineStr">
+        <is>
+          <t>PIX ENVIADO</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>Simone Bastos Gomes</t>
+        </is>
+      </c>
+      <c r="D46" s="9" t="n">
+        <v>1750</v>
+      </c>
+      <c r="E46" s="5" t="inlineStr">
+        <is>
+          <t>PIX P/ TERCEIROS</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>13/12/2025</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>APLICAÇÃO RDB</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>Investimento automático</t>
+        </is>
+      </c>
+      <c r="D47" s="9" t="n">
+        <v>5500</v>
+      </c>
+      <c r="E47" s="5" t="inlineStr">
+        <is>
+          <t>APLICAÇÃO RDB</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>09/02/2026</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t>BOLETO</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>GEAZI ASSIS DE SOUZA OLIVEIRA</t>
+        </is>
+      </c>
+      <c r="D48" s="9" t="n">
+        <v>195.5</v>
+      </c>
+      <c r="E48" s="5" t="inlineStr">
+        <is>
+          <t>PREFEITURA/CARTÓRIO</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>16/03/2026</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t>APLICAÇÃO RDB</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>Investimento automático</t>
+        </is>
+      </c>
+      <c r="D49" s="9" t="n">
+        <v>9600</v>
+      </c>
+      <c r="E49" s="5" t="inlineStr">
+        <is>
+          <t>APLICAÇÃO RDB</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>22/04/2026</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="inlineStr">
+        <is>
+          <t>APLICAÇÃO RDB</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>Investimento automático</t>
+        </is>
+      </c>
+      <c r="D50" s="9" t="n">
+        <v>2700</v>
+      </c>
+      <c r="E50" s="5" t="inlineStr">
+        <is>
+          <t>APLICAÇÃO RDB</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>19/05/2026</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="inlineStr">
+        <is>
+          <t>APLICAÇÃO RDB</t>
+        </is>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>Investimento automático</t>
+        </is>
+      </c>
+      <c r="D51" s="9" t="n">
+        <v>2000</v>
+      </c>
+      <c r="E51" s="5" t="inlineStr">
+        <is>
+          <t>APLICAÇÃO RDB</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="C53" s="28" t="inlineStr">
+        <is>
+          <t>TOTAL GERAL</t>
+        </is>
+      </c>
+      <c r="D53" s="30" t="n">
+        <v>159793.45</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="31" t="inlineStr">
+        <is>
+          <t>RESUMO POR CATEGORIA</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="32" t="inlineStr">
+        <is>
+          <t>CATEGORIA</t>
+        </is>
+      </c>
+      <c r="B56" s="32" t="inlineStr">
+        <is>
+          <t>QTD</t>
+        </is>
+      </c>
+      <c r="C56" s="32" t="inlineStr">
+        <is>
+          <t>TOTAL (R$)</t>
+        </is>
+      </c>
+      <c r="D56" s="32" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t>HONORÁRIOS</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C57" s="33" t="n">
+        <v>15000</v>
+      </c>
+      <c r="D57" s="34" t="n">
+        <v>0.0938711818287921</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>TOPÓGRAFO</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="C58" s="33" t="n">
+        <v>28750</v>
+      </c>
+      <c r="D58" s="34" t="n">
+        <v>0.1799197651718515</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="5" t="inlineStr">
+        <is>
+          <t>PREFEITURA/CARTÓRIO</t>
+        </is>
+      </c>
+      <c r="B59" s="5" t="n">
         <v>7</v>
       </c>
-      <c r="C32" s="33" t="n">
+      <c r="C59" s="33" t="n">
+        <v>791.4400000000001</v>
+      </c>
+      <c r="D59" s="34" t="n">
+        <v>0.004952893876438615</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="5" t="inlineStr">
+        <is>
+          <t>PIX P/ TERCEIROS</t>
+        </is>
+      </c>
+      <c r="B60" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="C60" s="33" t="n">
         <v>10670.48</v>
       </c>
-      <c r="D32" s="34" t="n">
-        <v>0.1932640632674973</v>
+      <c r="D60" s="34" t="n">
+        <v>0.06677670455203263</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="5" t="inlineStr">
+        <is>
+          <t>APLICAÇÃO RDB</t>
+        </is>
+      </c>
+      <c r="B61" s="5" t="n">
+        <v>28</v>
+      </c>
+      <c r="C61" s="33" t="n">
+        <v>104581.53</v>
+      </c>
+      <c r="D61" s="34" t="n">
+        <v>0.6544794545708851</v>
       </c>
     </row>
   </sheetData>
@@ -6615,7 +7390,7 @@
     <row r="2">
       <c r="A2" s="35" t="inlineStr">
         <is>
-          <t>Aplicações RDB excluídas conforme solicitação</t>
+          <t>Inclui aplicações RDB e pagamentos</t>
         </is>
       </c>
     </row>
@@ -6663,14 +7438,14 @@
       <c r="C5" s="37" t="n">
         <v>9405.940000000001</v>
       </c>
-      <c r="D5" s="9" t="n">
-        <v>0</v>
+      <c r="D5" s="38" t="n">
+        <v>10800</v>
       </c>
       <c r="E5" s="33" t="n">
-        <v>9405.940000000001</v>
-      </c>
-      <c r="F5" s="38" t="n">
-        <v>594.0599999999995</v>
+        <v>20205.94</v>
+      </c>
+      <c r="F5" s="10" t="n">
+        <v>-10205.94</v>
       </c>
     </row>
     <row r="6">
@@ -6685,14 +7460,14 @@
       <c r="C6" s="37" t="n">
         <v>9000</v>
       </c>
-      <c r="D6" s="9" t="n">
-        <v>0</v>
+      <c r="D6" s="38" t="n">
+        <v>9594.16</v>
       </c>
       <c r="E6" s="33" t="n">
-        <v>9000</v>
-      </c>
-      <c r="F6" s="38" t="n">
-        <v>500</v>
+        <v>18594.16</v>
+      </c>
+      <c r="F6" s="10" t="n">
+        <v>-9094.16</v>
       </c>
     </row>
     <row r="7">
@@ -6707,14 +7482,14 @@
       <c r="C7" s="37" t="n">
         <v>35.36</v>
       </c>
-      <c r="D7" s="9" t="n">
-        <v>0</v>
+      <c r="D7" s="38" t="n">
+        <v>6000</v>
       </c>
       <c r="E7" s="33" t="n">
-        <v>35.36</v>
-      </c>
-      <c r="F7" s="38" t="n">
-        <v>9464.639999999999</v>
+        <v>6035.36</v>
+      </c>
+      <c r="F7" s="39" t="n">
+        <v>3464.64</v>
       </c>
     </row>
     <row r="8">
@@ -6729,14 +7504,14 @@
       <c r="C8" s="37" t="n">
         <v>5278.69</v>
       </c>
-      <c r="D8" s="9" t="n">
-        <v>0</v>
+      <c r="D8" s="38" t="n">
+        <v>8135.95</v>
       </c>
       <c r="E8" s="33" t="n">
-        <v>5278.69</v>
-      </c>
-      <c r="F8" s="38" t="n">
-        <v>3221.31</v>
+        <v>13414.64</v>
+      </c>
+      <c r="F8" s="10" t="n">
+        <v>-4914.639999999999</v>
       </c>
     </row>
     <row r="9">
@@ -6751,14 +7526,14 @@
       <c r="C9" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="D9" s="9" t="n">
-        <v>0</v>
+      <c r="D9" s="38" t="n">
+        <v>7250</v>
       </c>
       <c r="E9" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="F9" s="38" t="n">
-        <v>8250</v>
+        <v>7250</v>
+      </c>
+      <c r="F9" s="39" t="n">
+        <v>1000</v>
       </c>
     </row>
     <row r="10">
@@ -6779,7 +7554,7 @@
       <c r="E10" s="33" t="n">
         <v>0</v>
       </c>
-      <c r="F10" s="38" t="n">
+      <c r="F10" s="39" t="n">
         <v>6000</v>
       </c>
     </row>
@@ -6795,14 +7570,14 @@
       <c r="C11" s="37" t="n">
         <v>11900</v>
       </c>
-      <c r="D11" s="9" t="n">
-        <v>0</v>
+      <c r="D11" s="38" t="n">
+        <v>8500</v>
       </c>
       <c r="E11" s="33" t="n">
-        <v>11900</v>
+        <v>20400</v>
       </c>
       <c r="F11" s="10" t="n">
-        <v>-8900</v>
+        <v>-17400</v>
       </c>
     </row>
     <row r="12">
@@ -6817,14 +7592,14 @@
       <c r="C12" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="D12" s="9" t="n">
-        <v>0</v>
+      <c r="D12" s="38" t="n">
+        <v>4750</v>
       </c>
       <c r="E12" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="F12" s="38" t="n">
-        <v>4250</v>
+        <v>4750</v>
+      </c>
+      <c r="F12" s="10" t="n">
+        <v>-500</v>
       </c>
     </row>
     <row r="13">
@@ -6839,14 +7614,14 @@
       <c r="C13" s="37" t="n">
         <v>11900</v>
       </c>
-      <c r="D13" s="9" t="n">
-        <v>0</v>
+      <c r="D13" s="38" t="n">
+        <v>3250</v>
       </c>
       <c r="E13" s="33" t="n">
-        <v>11900</v>
+        <v>15150</v>
       </c>
       <c r="F13" s="10" t="n">
-        <v>-7900</v>
+        <v>-11150</v>
       </c>
     </row>
     <row r="14">
@@ -6861,14 +7636,14 @@
       <c r="C14" s="37" t="n">
         <v>3800</v>
       </c>
-      <c r="D14" s="9" t="n">
-        <v>0</v>
+      <c r="D14" s="38" t="n">
+        <v>2750</v>
       </c>
       <c r="E14" s="33" t="n">
-        <v>3800</v>
-      </c>
-      <c r="F14" s="38" t="n">
-        <v>700</v>
+        <v>6550</v>
+      </c>
+      <c r="F14" s="10" t="n">
+        <v>-2050</v>
       </c>
     </row>
     <row r="15">
@@ -6889,7 +7664,7 @@
       <c r="E15" s="33" t="n">
         <v>0</v>
       </c>
-      <c r="F15" s="38" t="n">
+      <c r="F15" s="39" t="n">
         <v>4500</v>
       </c>
     </row>
@@ -6905,14 +7680,14 @@
       <c r="C16" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="D16" s="9" t="n">
-        <v>0</v>
+      <c r="D16" s="38" t="n">
+        <v>10251.42</v>
       </c>
       <c r="E16" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="F16" s="38" t="n">
-        <v>4000</v>
+        <v>10251.42</v>
+      </c>
+      <c r="F16" s="10" t="n">
+        <v>-6251.42</v>
       </c>
     </row>
     <row r="17">
@@ -6933,7 +7708,7 @@
       <c r="E17" s="33" t="n">
         <v>1750</v>
       </c>
-      <c r="F17" s="38" t="n">
+      <c r="F17" s="39" t="n">
         <v>1750</v>
       </c>
     </row>
@@ -6949,14 +7724,14 @@
       <c r="C18" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="D18" s="9" t="n">
-        <v>0</v>
+      <c r="D18" s="38" t="n">
+        <v>6000</v>
       </c>
       <c r="E18" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="F18" s="38" t="n">
-        <v>3250</v>
+        <v>6000</v>
+      </c>
+      <c r="F18" s="10" t="n">
+        <v>-2750</v>
       </c>
     </row>
     <row r="19">
@@ -6971,14 +7746,14 @@
       <c r="C19" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="D19" s="9" t="n">
-        <v>0</v>
+      <c r="D19" s="38" t="n">
+        <v>1000</v>
       </c>
       <c r="E19" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="F19" s="38" t="n">
-        <v>3250</v>
+        <v>1000</v>
+      </c>
+      <c r="F19" s="39" t="n">
+        <v>2250</v>
       </c>
     </row>
     <row r="20">
@@ -6993,14 +7768,14 @@
       <c r="C20" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="D20" s="9" t="n">
-        <v>0</v>
+      <c r="D20" s="38" t="n">
+        <v>6500</v>
       </c>
       <c r="E20" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="F20" s="38" t="n">
-        <v>4250</v>
+        <v>6500</v>
+      </c>
+      <c r="F20" s="10" t="n">
+        <v>-2250</v>
       </c>
     </row>
     <row r="21">
@@ -7021,7 +7796,7 @@
       <c r="E21" s="33" t="n">
         <v>1946.43</v>
       </c>
-      <c r="F21" s="38" t="n">
+      <c r="F21" s="39" t="n">
         <v>2053.57</v>
       </c>
     </row>
@@ -7037,14 +7812,14 @@
       <c r="C22" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="D22" s="9" t="n">
-        <v>0</v>
+      <c r="D22" s="38" t="n">
+        <v>5500</v>
       </c>
       <c r="E22" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="F22" s="38" t="n">
-        <v>3250</v>
+        <v>5500</v>
+      </c>
+      <c r="F22" s="10" t="n">
+        <v>-2250</v>
       </c>
     </row>
     <row r="23">
@@ -7065,7 +7840,7 @@
       <c r="E23" s="33" t="n">
         <v>0</v>
       </c>
-      <c r="F23" s="38" t="n">
+      <c r="F23" s="39" t="n">
         <v>2750</v>
       </c>
     </row>
@@ -7087,7 +7862,7 @@
       <c r="E24" s="33" t="n">
         <v>195.5</v>
       </c>
-      <c r="F24" s="38" t="n">
+      <c r="F24" s="39" t="n">
         <v>3554.5</v>
       </c>
     </row>
@@ -7103,14 +7878,14 @@
       <c r="C25" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="D25" s="9" t="n">
-        <v>0</v>
+      <c r="D25" s="38" t="n">
+        <v>9600</v>
       </c>
       <c r="E25" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="F25" s="38" t="n">
-        <v>3000</v>
+        <v>9600</v>
+      </c>
+      <c r="F25" s="10" t="n">
+        <v>-6600</v>
       </c>
     </row>
     <row r="26">
@@ -7125,14 +7900,14 @@
       <c r="C26" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="D26" s="9" t="n">
-        <v>0</v>
+      <c r="D26" s="38" t="n">
+        <v>2700</v>
       </c>
       <c r="E26" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="F26" s="38" t="n">
-        <v>2000</v>
+        <v>2700</v>
+      </c>
+      <c r="F26" s="10" t="n">
+        <v>-700</v>
       </c>
     </row>
     <row r="27">
@@ -7147,14 +7922,14 @@
       <c r="C27" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="D27" s="9" t="n">
-        <v>0</v>
+      <c r="D27" s="38" t="n">
+        <v>2000</v>
       </c>
       <c r="E27" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="F27" s="38" t="n">
-        <v>2530</v>
+        <v>2000</v>
+      </c>
+      <c r="F27" s="39" t="n">
+        <v>530</v>
       </c>
     </row>
     <row r="28">
@@ -7175,7 +7950,7 @@
       <c r="E28" s="33" t="n">
         <v>0</v>
       </c>
-      <c r="F28" s="38" t="n">
+      <c r="F28" s="39" t="n">
         <v>1250</v>
       </c>
     </row>
@@ -7192,13 +7967,13 @@
         <v>55211.92000000001</v>
       </c>
       <c r="D30" s="20" t="n">
-        <v>0</v>
+        <v>104581.53</v>
       </c>
       <c r="E30" s="20" t="n">
-        <v>55211.92000000001</v>
+        <v>159793.45</v>
       </c>
       <c r="F30" s="20" t="n">
-        <v>57568.07999999999</v>
+        <v>-47013.45</v>
       </c>
     </row>
   </sheetData>
@@ -14005,7 +14780,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="39" t="inlineStr">
+      <c r="A1" s="40" t="inlineStr">
         <is>
           <t>PONTOS DE ATENÇÃO E DIVERGÊNCIAS</t>
         </is>
@@ -14049,7 +14824,7 @@
           <t>NUNCA PAGOU. R$ 0 de R$ 12.000.</t>
         </is>
       </c>
-      <c r="D4" s="40" t="inlineStr">
+      <c r="D4" s="41" t="inlineStr">
         <is>
           <t>INADIMPLENTE</t>
         </is>
@@ -14071,7 +14846,7 @@
           <t>Parou de pagar após NOV/2024. Saldo devedor alto.</t>
         </is>
       </c>
-      <c r="D5" s="40" t="inlineStr">
+      <c r="D5" s="41" t="inlineStr">
         <is>
           <t>INADIMPLENTE</t>
         </is>
@@ -14093,7 +14868,7 @@
           <t>Parou de pagar após OUT/2024.</t>
         </is>
       </c>
-      <c r="D6" s="40" t="inlineStr">
+      <c r="D6" s="41" t="inlineStr">
         <is>
           <t>INADIMPLENTE</t>
         </is>
@@ -14115,7 +14890,7 @@
           <t>Parou de pagar após MAR/2025.</t>
         </is>
       </c>
-      <c r="D7" s="40" t="inlineStr">
+      <c r="D7" s="41" t="inlineStr">
         <is>
           <t>INADIMPLENTE</t>
         </is>
@@ -14137,7 +14912,7 @@
           <t>Último pagamento JUN/2025.</t>
         </is>
       </c>
-      <c r="D8" s="40" t="inlineStr">
+      <c r="D8" s="41" t="inlineStr">
         <is>
           <t>INADIMPLENTE</t>
         </is>
@@ -14159,7 +14934,7 @@
           <t>Pagamentos irregulares. Último SET/2025.</t>
         </is>
       </c>
-      <c r="D9" s="40" t="inlineStr">
+      <c r="D9" s="41" t="inlineStr">
         <is>
           <t>INADIMPLENTE</t>
         </is>
@@ -14181,7 +14956,7 @@
           <t>Pagou apenas JUL/24. Eduardo N. Lobato continua pagando.</t>
         </is>
       </c>
-      <c r="D10" s="41" t="inlineStr">
+      <c r="D10" s="42" t="inlineStr">
         <is>
           <t>ATENÇÃO</t>
         </is>
@@ -14203,7 +14978,7 @@
           <t>Pagamentos irregulares (R$ 1.000 esporádicos). Sem pagto desde FEV/26.</t>
         </is>
       </c>
-      <c r="D11" s="41" t="inlineStr">
+      <c r="D11" s="42" t="inlineStr">
         <is>
           <t>ATENÇÃO</t>
         </is>
@@ -14225,7 +15000,7 @@
           <t>Pagou R$ 30 em 26/05/2026 (habitual R$ 250). Verificar.</t>
         </is>
       </c>
-      <c r="D12" s="41" t="inlineStr">
+      <c r="D12" s="42" t="inlineStr">
         <is>
           <t>ATENÇÃO</t>
         </is>
@@ -14247,7 +15022,7 @@
           <t>ABR/26: pagou R$ 500 (habitual R$ 750). Pagam pelos mesmos lotes.</t>
         </is>
       </c>
-      <c r="D13" s="41" t="inlineStr">
+      <c r="D13" s="42" t="inlineStr">
         <is>
           <t>ATENÇÃO</t>
         </is>
@@ -14269,7 +15044,7 @@
           <t>Parcela reduzida. Pagou MAR/26 e parou.</t>
         </is>
       </c>
-      <c r="D14" s="41" t="inlineStr">
+      <c r="D14" s="42" t="inlineStr">
         <is>
           <t>ATENÇÃO</t>
         </is>
@@ -14291,7 +15066,7 @@
           <t>Sem pagamento ABR/26 e JUN/26.</t>
         </is>
       </c>
-      <c r="D15" s="41" t="inlineStr">
+      <c r="D15" s="42" t="inlineStr">
         <is>
           <t>ATENÇÃO</t>
         </is>
@@ -14313,7 +15088,7 @@
           <t>Pagamentos irregulares.</t>
         </is>
       </c>
-      <c r="D16" s="41" t="inlineStr">
+      <c r="D16" s="42" t="inlineStr">
         <is>
           <t>ATENÇÃO</t>
         </is>
@@ -14335,7 +15110,7 @@
           <t>Consistente R$ 500/mês. Sem JUN/26 (extrato até 11/06).</t>
         </is>
       </c>
-      <c r="D17" s="42" t="inlineStr">
+      <c r="D17" s="43" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -14344,4 +15119,1384 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F75"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>CONCILIAÇÃO - EXTRATO CAIXINHAS RDB vs EXTRATO BANCÁRIO</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="44" t="inlineStr">
+        <is>
+          <t>Período: MAI/2025 a JUN/2026 | Nu Financeira S.A. | Saldo final: R$ 68.284,51</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="45" t="inlineStr">
+        <is>
+          <t>DATA</t>
+        </is>
+      </c>
+      <c r="B4" s="45" t="inlineStr">
+        <is>
+          <t>MOVIMENTAÇÃO</t>
+        </is>
+      </c>
+      <c r="C4" s="45" t="inlineStr">
+        <is>
+          <t>RENDIMENTO (R$)</t>
+        </is>
+      </c>
+      <c r="D4" s="45" t="inlineStr">
+        <is>
+          <t>VALOR APLICADO (R$)</t>
+        </is>
+      </c>
+      <c r="E4" s="45" t="inlineStr">
+        <is>
+          <t>SALDO ACUMULADO (R$)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>31/05/2025</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Rendimento</t>
+        </is>
+      </c>
+      <c r="C5" s="46" t="n">
+        <v>247.14</v>
+      </c>
+      <c r="D5" s="5" t="n"/>
+      <c r="E5" s="33" t="n">
+        <v>247.14</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>15/06/2025</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Compra por aplicação</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="n"/>
+      <c r="D6" s="46" t="n">
+        <v>10251.42</v>
+      </c>
+      <c r="E6" s="33" t="n">
+        <v>10498.56</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>30/06/2025</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Rendimento</t>
+        </is>
+      </c>
+      <c r="C7" s="46" t="n">
+        <v>205.7</v>
+      </c>
+      <c r="D7" s="5" t="n"/>
+      <c r="E7" s="33" t="n">
+        <v>10704.26</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>01/07/2025</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Resgate</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="n"/>
+      <c r="D8" s="47" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E8" s="33" t="n">
+        <v>9704.26</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>31/07/2025</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Rendimento</t>
+        </is>
+      </c>
+      <c r="C9" s="46" t="n">
+        <v>418.99</v>
+      </c>
+      <c r="D9" s="5" t="n"/>
+      <c r="E9" s="33" t="n">
+        <v>10123.25</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>08/08/2025</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Compra por aplicação</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="n"/>
+      <c r="D10" s="46" t="n">
+        <v>3750</v>
+      </c>
+      <c r="E10" s="33" t="n">
+        <v>13873.25</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>11/08/2025</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Compra por aplicação</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="n"/>
+      <c r="D11" s="46" t="n">
+        <v>2250</v>
+      </c>
+      <c r="E11" s="33" t="n">
+        <v>16123.25</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>31/08/2025</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Rendimento</t>
+        </is>
+      </c>
+      <c r="C12" s="46" t="n">
+        <v>361.46</v>
+      </c>
+      <c r="D12" s="5" t="n"/>
+      <c r="E12" s="33" t="n">
+        <v>16484.71</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>08/09/2025</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Compra por aplicação</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="n"/>
+      <c r="D13" s="46" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E13" s="33" t="n">
+        <v>17484.71</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>30/09/2025</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Rendimento</t>
+        </is>
+      </c>
+      <c r="C14" s="46" t="n">
+        <v>471.49</v>
+      </c>
+      <c r="D14" s="5" t="n"/>
+      <c r="E14" s="33" t="n">
+        <v>17956.2</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>13/10/2025</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Compra por aplicação</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="n"/>
+      <c r="D15" s="46" t="n">
+        <v>6500</v>
+      </c>
+      <c r="E15" s="33" t="n">
+        <v>24456.2</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>31/10/2025</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Rendimento</t>
+        </is>
+      </c>
+      <c r="C16" s="46" t="n">
+        <v>486.89</v>
+      </c>
+      <c r="D16" s="5" t="n"/>
+      <c r="E16" s="33" t="n">
+        <v>24943.09</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>10/11/2025</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Resgate</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="n"/>
+      <c r="D17" s="47" t="n">
+        <v>500</v>
+      </c>
+      <c r="E17" s="33" t="n">
+        <v>24443.09</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>30/11/2025</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Rendimento</t>
+        </is>
+      </c>
+      <c r="C18" s="46" t="n">
+        <v>534.14</v>
+      </c>
+      <c r="D18" s="5" t="n"/>
+      <c r="E18" s="33" t="n">
+        <v>24977.23</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>13/12/2025</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Compra por aplicação</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="n"/>
+      <c r="D19" s="46" t="n">
+        <v>5500</v>
+      </c>
+      <c r="E19" s="33" t="n">
+        <v>30477.23</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>31/12/2025</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Rendimento</t>
+        </is>
+      </c>
+      <c r="C20" s="46" t="n">
+        <v>517.86</v>
+      </c>
+      <c r="D20" s="5" t="n"/>
+      <c r="E20" s="33" t="n">
+        <v>30995.09</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>31/01/2026</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Rendimento</t>
+        </is>
+      </c>
+      <c r="C21" s="46" t="n">
+        <v>649.9400000000001</v>
+      </c>
+      <c r="D21" s="5" t="n"/>
+      <c r="E21" s="33" t="n">
+        <v>31645.03</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>28/02/2026</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Rendimento</t>
+        </is>
+      </c>
+      <c r="C22" s="46" t="n">
+        <v>509.98</v>
+      </c>
+      <c r="D22" s="5" t="n"/>
+      <c r="E22" s="33" t="n">
+        <v>32155.01</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>16/03/2026</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Compra por aplicação</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="n"/>
+      <c r="D23" s="46" t="n">
+        <v>9600</v>
+      </c>
+      <c r="E23" s="33" t="n">
+        <v>41755.01</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>31/03/2026</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>Rendimento</t>
+        </is>
+      </c>
+      <c r="C24" s="46" t="n">
+        <v>597.8</v>
+      </c>
+      <c r="D24" s="5" t="n"/>
+      <c r="E24" s="33" t="n">
+        <v>42352.81</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>22/04/2026</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>Compra por aplicação</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="n"/>
+      <c r="D25" s="46" t="n">
+        <v>2700</v>
+      </c>
+      <c r="E25" s="33" t="n">
+        <v>45052.81</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>30/04/2026</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Rendimento</t>
+        </is>
+      </c>
+      <c r="C26" s="46" t="n">
+        <v>733.22</v>
+      </c>
+      <c r="D26" s="5" t="n"/>
+      <c r="E26" s="33" t="n">
+        <v>45786.03</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>19/05/2026</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Compra por aplicação</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="n"/>
+      <c r="D27" s="46" t="n">
+        <v>2000</v>
+      </c>
+      <c r="E27" s="33" t="n">
+        <v>47786.03</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>31/05/2026</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Rendimento</t>
+        </is>
+      </c>
+      <c r="C28" s="46" t="n">
+        <v>744.97</v>
+      </c>
+      <c r="D28" s="5" t="n"/>
+      <c r="E28" s="33" t="n">
+        <v>48531</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>11/06/2026</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>Rendimento</t>
+        </is>
+      </c>
+      <c r="C29" s="46" t="n">
+        <v>247.26</v>
+      </c>
+      <c r="D29" s="5" t="n"/>
+      <c r="E29" s="33" t="n">
+        <v>48778.26</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="17" t="inlineStr">
+        <is>
+          <t>TOTAIS</t>
+        </is>
+      </c>
+      <c r="B31" s="18" t="n"/>
+      <c r="C31" s="48" t="n">
+        <v>6726.84</v>
+      </c>
+      <c r="D31" s="48" t="n">
+        <v>43551.42</v>
+      </c>
+      <c r="E31" s="49" t="n">
+        <v>48778.26</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="31" t="inlineStr">
+        <is>
+          <t>RESUMO CAIXINHAS RDB</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="50" t="inlineStr">
+        <is>
+          <t>Total aplicado (compras)</t>
+        </is>
+      </c>
+      <c r="B34" s="51" t="n">
+        <v>43551.42</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="50" t="inlineStr">
+        <is>
+          <t>Total resgatado</t>
+        </is>
+      </c>
+      <c r="B35" s="51" t="n">
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="50" t="inlineStr">
+        <is>
+          <t>Total rendimentos</t>
+        </is>
+      </c>
+      <c r="B36" s="51" t="n">
+        <v>6726.840000000001</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="50" t="inlineStr">
+        <is>
+          <t>Saldo final caixinhas (extrato)</t>
+        </is>
+      </c>
+      <c r="B37" s="51" t="n">
+        <v>68284.50999999999</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="50" t="inlineStr">
+        <is>
+          <t>Saldo calculado</t>
+        </is>
+      </c>
+      <c r="B38" s="51" t="n">
+        <v>48778.26</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="50" t="inlineStr">
+        <is>
+          <t>Diferença</t>
+        </is>
+      </c>
+      <c r="B39" s="52" t="n">
+        <v>19506.25</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="53" t="inlineStr">
+        <is>
+          <t>CONCILIAÇÃO: EXTRATO BANCÁRIO vs CAIXINHAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>Verifica se cada "Aplicação RDB" do extrato bancário bate com "Compra por aplicação" do extrato de caixinhas</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="54" t="inlineStr">
+        <is>
+          <t>DATA EXTRATO BANCÁRIO</t>
+        </is>
+      </c>
+      <c r="B44" s="54" t="inlineStr">
+        <is>
+          <t>VALOR EXTRATO (R$)</t>
+        </is>
+      </c>
+      <c r="C44" s="54" t="inlineStr">
+        <is>
+          <t>DATA CAIXINHAS</t>
+        </is>
+      </c>
+      <c r="D44" s="54" t="inlineStr">
+        <is>
+          <t>VALOR CAIXINHAS (R$)</t>
+        </is>
+      </c>
+      <c r="E44" s="54" t="inlineStr">
+        <is>
+          <t>STATUS</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>15/07/2024</t>
+        </is>
+      </c>
+      <c r="B45" s="9" t="n">
+        <v>8800</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E45" s="55" t="inlineStr">
+        <is>
+          <t>NÃO ENCONTRADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>16/07/2024</t>
+        </is>
+      </c>
+      <c r="B46" s="9" t="n">
+        <v>500</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D46" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E46" s="55" t="inlineStr">
+        <is>
+          <t>NÃO ENCONTRADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>21/07/2024</t>
+        </is>
+      </c>
+      <c r="B47" s="9" t="n">
+        <v>1500</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D47" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E47" s="55" t="inlineStr">
+        <is>
+          <t>NÃO ENCONTRADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>06/08/2024</t>
+        </is>
+      </c>
+      <c r="B48" s="9" t="n">
+        <v>594.16</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D48" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E48" s="55" t="inlineStr">
+        <is>
+          <t>NÃO ENCONTRADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>11/08/2024</t>
+        </is>
+      </c>
+      <c r="B49" s="9" t="n">
+        <v>6000</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D49" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E49" s="55" t="inlineStr">
+        <is>
+          <t>NÃO ENCONTRADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>13/08/2024</t>
+        </is>
+      </c>
+      <c r="B50" s="9" t="n">
+        <v>500</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D50" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E50" s="55" t="inlineStr">
+        <is>
+          <t>NÃO ENCONTRADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>18/08/2024</t>
+        </is>
+      </c>
+      <c r="B51" s="9" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>08/09/2025</t>
+        </is>
+      </c>
+      <c r="D51" s="9" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E51" s="56" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>25/08/2024</t>
+        </is>
+      </c>
+      <c r="B52" s="9" t="n">
+        <v>1500</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D52" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E52" s="55" t="inlineStr">
+        <is>
+          <t>NÃO ENCONTRADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>16/09/2024</t>
+        </is>
+      </c>
+      <c r="B53" s="9" t="n">
+        <v>6000</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D53" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E53" s="55" t="inlineStr">
+        <is>
+          <t>NÃO ENCONTRADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>13/10/2024</t>
+        </is>
+      </c>
+      <c r="B54" s="9" t="n">
+        <v>7635.95</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D54" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E54" s="55" t="inlineStr">
+        <is>
+          <t>NÃO ENCONTRADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>30/10/2024</t>
+        </is>
+      </c>
+      <c r="B55" s="9" t="n">
+        <v>500</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D55" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E55" s="55" t="inlineStr">
+        <is>
+          <t>NÃO ENCONTRADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>24/11/2024</t>
+        </is>
+      </c>
+      <c r="B56" s="9" t="n">
+        <v>7250</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D56" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E56" s="55" t="inlineStr">
+        <is>
+          <t>NÃO ENCONTRADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t>06/01/2025</t>
+        </is>
+      </c>
+      <c r="B57" s="9" t="n">
+        <v>7000</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D57" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E57" s="55" t="inlineStr">
+        <is>
+          <t>NÃO ENCONTRADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>07/01/2025</t>
+        </is>
+      </c>
+      <c r="B58" s="9" t="n">
+        <v>250</v>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D58" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E58" s="55" t="inlineStr">
+        <is>
+          <t>NÃO ENCONTRADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="5" t="inlineStr">
+        <is>
+          <t>12/01/2025</t>
+        </is>
+      </c>
+      <c r="B59" s="9" t="n">
+        <v>1250</v>
+      </c>
+      <c r="C59" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D59" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E59" s="55" t="inlineStr">
+        <is>
+          <t>NÃO ENCONTRADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="5" t="inlineStr">
+        <is>
+          <t>02/02/2025</t>
+        </is>
+      </c>
+      <c r="B60" s="9" t="n">
+        <v>1500</v>
+      </c>
+      <c r="C60" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D60" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E60" s="55" t="inlineStr">
+        <is>
+          <t>NÃO ENCONTRADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="5" t="inlineStr">
+        <is>
+          <t>23/02/2025</t>
+        </is>
+      </c>
+      <c r="B61" s="9" t="n">
+        <v>3250</v>
+      </c>
+      <c r="C61" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D61" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E61" s="55" t="inlineStr">
+        <is>
+          <t>NÃO ENCONTRADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="5" t="inlineStr">
+        <is>
+          <t>16/03/2025</t>
+        </is>
+      </c>
+      <c r="B62" s="9" t="n">
+        <v>3250</v>
+      </c>
+      <c r="C62" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D62" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E62" s="55" t="inlineStr">
+        <is>
+          <t>NÃO ENCONTRADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="5" t="inlineStr">
+        <is>
+          <t>12/04/2025</t>
+        </is>
+      </c>
+      <c r="B63" s="9" t="n">
+        <v>2750</v>
+      </c>
+      <c r="C63" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D63" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E63" s="55" t="inlineStr">
+        <is>
+          <t>NÃO ENCONTRADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="5" t="inlineStr">
+        <is>
+          <t>15/06/2025</t>
+        </is>
+      </c>
+      <c r="B64" s="9" t="n">
+        <v>10251.42</v>
+      </c>
+      <c r="C64" s="5" t="inlineStr">
+        <is>
+          <t>15/06/2025</t>
+        </is>
+      </c>
+      <c r="D64" s="9" t="n">
+        <v>10251.42</v>
+      </c>
+      <c r="E64" s="56" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="5" t="inlineStr">
+        <is>
+          <t>08/08/2025</t>
+        </is>
+      </c>
+      <c r="B65" s="9" t="n">
+        <v>3750</v>
+      </c>
+      <c r="C65" s="5" t="inlineStr">
+        <is>
+          <t>08/08/2025</t>
+        </is>
+      </c>
+      <c r="D65" s="9" t="n">
+        <v>3750</v>
+      </c>
+      <c r="E65" s="56" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="5" t="inlineStr">
+        <is>
+          <t>11/08/2025</t>
+        </is>
+      </c>
+      <c r="B66" s="9" t="n">
+        <v>2250</v>
+      </c>
+      <c r="C66" s="5" t="inlineStr">
+        <is>
+          <t>11/08/2025</t>
+        </is>
+      </c>
+      <c r="D66" s="9" t="n">
+        <v>2250</v>
+      </c>
+      <c r="E66" s="56" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="5" t="inlineStr">
+        <is>
+          <t>08/09/2025</t>
+        </is>
+      </c>
+      <c r="B67" s="9" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C67" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D67" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E67" s="55" t="inlineStr">
+        <is>
+          <t>NÃO ENCONTRADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="5" t="inlineStr">
+        <is>
+          <t>12/10/2025</t>
+        </is>
+      </c>
+      <c r="B68" s="9" t="n">
+        <v>6500</v>
+      </c>
+      <c r="C68" s="5" t="inlineStr">
+        <is>
+          <t>13/10/2025</t>
+        </is>
+      </c>
+      <c r="D68" s="9" t="n">
+        <v>6500</v>
+      </c>
+      <c r="E68" s="56" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="5" t="inlineStr">
+        <is>
+          <t>13/12/2025</t>
+        </is>
+      </c>
+      <c r="B69" s="9" t="n">
+        <v>5500</v>
+      </c>
+      <c r="C69" s="5" t="inlineStr">
+        <is>
+          <t>13/12/2025</t>
+        </is>
+      </c>
+      <c r="D69" s="9" t="n">
+        <v>5500</v>
+      </c>
+      <c r="E69" s="56" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="5" t="inlineStr">
+        <is>
+          <t>16/03/2026</t>
+        </is>
+      </c>
+      <c r="B70" s="9" t="n">
+        <v>9600</v>
+      </c>
+      <c r="C70" s="5" t="inlineStr">
+        <is>
+          <t>16/03/2026</t>
+        </is>
+      </c>
+      <c r="D70" s="9" t="n">
+        <v>9600</v>
+      </c>
+      <c r="E70" s="56" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="5" t="inlineStr">
+        <is>
+          <t>22/04/2026</t>
+        </is>
+      </c>
+      <c r="B71" s="9" t="n">
+        <v>2700</v>
+      </c>
+      <c r="C71" s="5" t="inlineStr">
+        <is>
+          <t>22/04/2026</t>
+        </is>
+      </c>
+      <c r="D71" s="9" t="n">
+        <v>2700</v>
+      </c>
+      <c r="E71" s="56" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="5" t="inlineStr">
+        <is>
+          <t>19/05/2026</t>
+        </is>
+      </c>
+      <c r="B72" s="9" t="n">
+        <v>2000</v>
+      </c>
+      <c r="C72" s="5" t="inlineStr">
+        <is>
+          <t>19/05/2026</t>
+        </is>
+      </c>
+      <c r="D72" s="9" t="n">
+        <v>2000</v>
+      </c>
+      <c r="E72" s="56" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="57" t="inlineStr">
+        <is>
+          <t>TOTAL EXTRATO BANCÁRIO</t>
+        </is>
+      </c>
+      <c r="B74" s="48" t="n">
+        <v>104581.53</v>
+      </c>
+      <c r="C74" s="57" t="inlineStr">
+        <is>
+          <t>TOTAL CAIXINHAS</t>
+        </is>
+      </c>
+      <c r="D74" s="48" t="n">
+        <v>43551.42</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="58" t="inlineStr">
+        <is>
+          <t>DIFERENÇA</t>
+        </is>
+      </c>
+      <c r="B75" s="59" t="n">
+        <v>61030.11</v>
+      </c>
+      <c r="C75" s="60" t="inlineStr">
+        <is>
+          <t>DIVERGÊNCIA</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>